<commit_message>
adding and update files
</commit_message>
<xml_diff>
--- a/##RPS Biostatistika Teori (By Ferdycov).xlsx
+++ b/##RPS Biostatistika Teori (By Ferdycov).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\02. Dosen\##MATERI BIOSTAT\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADMIN\Downloads\#Bootcamp\biostatistic_medical_record\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5B8F693-A909-4B29-8FC2-76600782DD35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CE68F86-721D-4671-8CC2-6DF267D7DA93}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{CF258F82-91C1-4CE6-A45F-31BD05A0E31D}"/>
+    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12450" xr2:uid="{CF258F82-91C1-4CE6-A45F-31BD05A0E31D}"/>
   </bookViews>
   <sheets>
     <sheet name="rps ferdy mandiri" sheetId="1" r:id="rId1"/>
@@ -621,17 +621,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E883A153-C4CB-451A-A6F7-6E11CED65E25}">
   <dimension ref="B2:N25"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="8" style="10" customWidth="1"/>
     <col min="3" max="3" width="21" customWidth="1"/>
-    <col min="4" max="4" width="60.44140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="50.33203125" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="60.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="50.28515625" hidden="1" customWidth="1"/>
     <col min="6" max="6" width="18" hidden="1" customWidth="1"/>
-    <col min="7" max="7" width="3.21875" customWidth="1"/>
+    <col min="7" max="7" width="3.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B2" s="7" t="s">
         <v>0</v>
       </c>
@@ -639,7 +639,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B3" s="3" t="s">
         <v>2</v>
       </c>
@@ -647,7 +647,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B4" s="3" t="s">
         <v>4</v>
       </c>
@@ -655,7 +655,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B5" s="3" t="s">
         <v>6</v>
       </c>
@@ -663,7 +663,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B6" s="3" t="s">
         <v>8</v>
       </c>
@@ -671,7 +671,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B7" s="3" t="s">
         <v>9</v>
       </c>
@@ -679,7 +679,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B8" s="3" t="s">
         <v>11</v>
       </c>
@@ -687,7 +687,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B9" s="8" t="s">
         <v>13</v>
       </c>
@@ -713,7 +713,7 @@
       <c r="M9" s="12"/>
       <c r="N9" s="12"/>
     </row>
-    <row r="10" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B10" s="9">
         <v>1</v>
       </c>
@@ -737,7 +737,7 @@
       <c r="M10" s="12"/>
       <c r="N10" s="12"/>
     </row>
-    <row r="11" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B11" s="9">
         <v>2</v>
       </c>
@@ -761,7 +761,7 @@
       <c r="M11" s="12"/>
       <c r="N11" s="12"/>
     </row>
-    <row r="12" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B12" s="9">
         <v>3</v>
       </c>
@@ -785,7 +785,7 @@
       <c r="M12" s="12"/>
       <c r="N12" s="12"/>
     </row>
-    <row r="13" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B13" s="9">
         <v>4</v>
       </c>
@@ -809,7 +809,7 @@
       <c r="M13" s="12"/>
       <c r="N13" s="12"/>
     </row>
-    <row r="14" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B14" s="9">
         <v>5</v>
       </c>
@@ -833,14 +833,14 @@
       <c r="M14" s="12"/>
       <c r="N14" s="12"/>
     </row>
-    <row r="15" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B15" s="9">
         <v>6</v>
       </c>
       <c r="C15" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="D15" s="5" t="s">
+      <c r="D15" s="11" t="s">
         <v>54</v>
       </c>
       <c r="E15" s="5" t="s">
@@ -857,7 +857,7 @@
       <c r="M15" s="12"/>
       <c r="N15" s="12"/>
     </row>
-    <row r="16" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B16" s="9">
         <v>7</v>
       </c>
@@ -881,7 +881,7 @@
       <c r="M16" s="12"/>
       <c r="N16" s="12"/>
     </row>
-    <row r="17" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B17" s="9">
         <v>8</v>
       </c>
@@ -905,7 +905,7 @@
       <c r="M17" s="12"/>
       <c r="N17" s="12"/>
     </row>
-    <row r="18" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B18" s="9">
         <v>9</v>
       </c>
@@ -929,7 +929,7 @@
       <c r="M18" s="12"/>
       <c r="N18" s="12"/>
     </row>
-    <row r="19" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B19" s="9">
         <v>10</v>
       </c>
@@ -953,7 +953,7 @@
       <c r="M19" s="12"/>
       <c r="N19" s="12"/>
     </row>
-    <row r="20" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B20" s="9">
         <v>11</v>
       </c>
@@ -977,7 +977,7 @@
       <c r="M20" s="12"/>
       <c r="N20" s="12"/>
     </row>
-    <row r="21" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B21" s="9">
         <v>12</v>
       </c>
@@ -1001,7 +1001,7 @@
       <c r="M21" s="12"/>
       <c r="N21" s="12"/>
     </row>
-    <row r="22" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B22" s="9">
         <v>13</v>
       </c>
@@ -1025,7 +1025,7 @@
       <c r="M22" s="12"/>
       <c r="N22" s="12"/>
     </row>
-    <row r="23" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B23" s="9">
         <v>14</v>
       </c>
@@ -1045,7 +1045,7 @@
       <c r="M23" s="12"/>
       <c r="N23" s="12"/>
     </row>
-    <row r="24" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B24" s="9">
         <v>15</v>
       </c>
@@ -1065,7 +1065,7 @@
       <c r="M24" s="12"/>
       <c r="N24" s="12"/>
     </row>
-    <row r="25" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B25" s="9">
         <v>16</v>
       </c>
@@ -1094,21 +1094,21 @@
     <mergeCell ref="H9:N25"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BAF3FC1C-2836-4717-9A56-B373103167AD}">
   <dimension ref="B2:G18"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="5.33203125" customWidth="1"/>
-    <col min="3" max="3" width="38.5546875" customWidth="1"/>
-    <col min="4" max="4" width="44.6640625" customWidth="1"/>
+    <col min="1" max="1" width="5.28515625" customWidth="1"/>
+    <col min="3" max="3" width="38.5703125" customWidth="1"/>
+    <col min="4" max="4" width="44.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">
         <v>13</v>
       </c>
@@ -1126,7 +1126,7 @@
       </c>
       <c r="G2" s="1"/>
     </row>
-    <row r="3" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3" s="2">
         <v>1</v>
       </c>
@@ -1144,7 +1144,7 @@
       </c>
       <c r="G3" s="2"/>
     </row>
-    <row r="4" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B4" s="2">
         <v>2</v>
       </c>
@@ -1162,7 +1162,7 @@
       </c>
       <c r="G4" s="2"/>
     </row>
-    <row r="5" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B5" s="2">
         <v>3</v>
       </c>
@@ -1180,7 +1180,7 @@
       </c>
       <c r="G5" s="2"/>
     </row>
-    <row r="6" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B6" s="2">
         <v>4</v>
       </c>
@@ -1198,7 +1198,7 @@
       </c>
       <c r="G6" s="2"/>
     </row>
-    <row r="7" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B7" s="2">
         <v>5</v>
       </c>
@@ -1216,7 +1216,7 @@
       </c>
       <c r="G7" s="2"/>
     </row>
-    <row r="8" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B8" s="2">
         <v>6</v>
       </c>
@@ -1234,7 +1234,7 @@
       </c>
       <c r="G8" s="2"/>
     </row>
-    <row r="9" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B9" s="2">
         <v>7</v>
       </c>
@@ -1252,7 +1252,7 @@
       </c>
       <c r="G9" s="2"/>
     </row>
-    <row r="10" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B10" s="2">
         <v>8</v>
       </c>
@@ -1270,7 +1270,7 @@
       </c>
       <c r="G10" s="2"/>
     </row>
-    <row r="11" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B11" s="2">
         <v>9</v>
       </c>
@@ -1288,7 +1288,7 @@
       </c>
       <c r="G11" s="2"/>
     </row>
-    <row r="12" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B12" s="2">
         <v>10</v>
       </c>
@@ -1306,7 +1306,7 @@
       </c>
       <c r="G12" s="2"/>
     </row>
-    <row r="13" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B13" s="2">
         <v>11</v>
       </c>
@@ -1324,7 +1324,7 @@
       </c>
       <c r="G13" s="2"/>
     </row>
-    <row r="14" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B14" s="2">
         <v>12</v>
       </c>
@@ -1342,7 +1342,7 @@
       </c>
       <c r="G14" s="2"/>
     </row>
-    <row r="15" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B15" s="2">
         <v>13</v>
       </c>
@@ -1360,7 +1360,7 @@
       </c>
       <c r="G15" s="2"/>
     </row>
-    <row r="16" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B16" s="2">
         <v>14</v>
       </c>
@@ -1371,7 +1371,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="17" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B17" s="2">
         <v>15</v>
       </c>
@@ -1385,7 +1385,7 @@
       <c r="F17" s="2"/>
       <c r="G17" s="2"/>
     </row>
-    <row r="18" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B18" s="2">
         <v>16</v>
       </c>

</xml_diff>

<commit_message>
adding & update files
</commit_message>
<xml_diff>
--- a/##RPS Biostatistika Teori (By Ferdycov).xlsx
+++ b/##RPS Biostatistika Teori (By Ferdycov).xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\02. Dosen\##MATERI BIOSTAT\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ACER\Desktop\HOBiostatistics\biostatistic_medical_record\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5B8F693-A909-4B29-8FC2-76600782DD35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDBEB6D4-7134-480A-AD16-E6254CA76BC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{CF258F82-91C1-4CE6-A45F-31BD05A0E31D}"/>
   </bookViews>
@@ -211,7 +211,8 @@
     <t>uji regresi</t>
   </si>
   <si>
-    <t>buatkan saya outline materi kuliah dengan topik : Central tendency. Buat dengan gaya akademis + daftar pustakanya. Buat dalam format quarto output PDF (urutannya : Pengantar/Pendahuluan, central tedency berisi definisi+kegunaannya+formula+cara menghitung + contoh di rekam medis + perbedaan masing masing central tendency, Latihan Soal, Kesimpulan, Daftar pustaka)</t>
+    <t>buatkan saya outline materi kuliah dengan topik : Central tendency. Buat dengan gaya akademis + daftar pustakanya. Buat dalam format quarto output PDF (urutannya : Pengantar/Pendahuluan, central tedency berisi definisi+kegunaannya+formula+cara menghitung + contoh di rekam medis + perbedaan masing masing central tendency, Latihan Soal, Kesimpulan, Daftar pustaka)
+buatkan saya outline materi kuliah dengan topik : Central tendency. Buat dengan gaya akademis + daftar pustakanya. Buat dalam format quarto output PDF (urutannya : Pengantar/Pendahuluan, dispersion berisi definisi+kegunaannya+formula+cara menghitung + contoh di rekam medis + perbedaan masing masing dispersion, Latihan Soal, Kesimpulan, Daftar pustaka)</t>
   </si>
 </sst>
 </file>
@@ -303,7 +304,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>

</xml_diff>